<commit_message>
style: mejora layout y estética de hojas de datos DTS
- Amplía tablas de A:F a A:O para coincidir con encabezado corporativo.
- Separa notas numeradas (6.1, 6.2, ...) en párrafos individuales.
- Aplica estilo cursivo/gris a notas numeradas.
- Incluye imágenes de referencia y curva en DTS-001.
- Recompila y emite 8 entregables actualizados.
- Actualiza contexto, vault y task/todo.md.
</commit_message>
<xml_diff>
--- a/Emisiones/3.0 HV-HOJAS DE DATOS/P2437-HV-DTS-001 REV0.xlsx
+++ b/Emisiones/3.0 HV-HOJAS DE DATOS/P2437-HV-DTS-001 REV0.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.00000000000000"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -146,6 +146,11 @@
       <b val="1"/>
       <color rgb="001F4E78"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00404040"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
@@ -337,7 +342,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
@@ -488,10 +493,13 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -683,7 +691,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId1"/>
+        <a:blip r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -724,7 +732,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill rotWithShape="1">
-        <a:blip r:embed="rId2"/>
+        <a:blip r:embed="rId4"/>
         <a:srcRect l="4540" t="12476" r="4665" b="12920"/>
         <a:stretch>
           <a:fillRect/>
@@ -745,6 +753,56 @@
     </pic>
     <clientData/>
   </twoCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>109</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5715000" cy="3810000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>130</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5715000" cy="3810000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -3218,7 +3276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O121"/>
+  <dimension ref="A1:O108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30.61328125" customWidth="1" min="1" max="1"/>
@@ -3450,15 +3508,24 @@
           <t>Campo</t>
         </is>
       </c>
-      <c r="B10" s="59" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
+      <c r="B10" s="59" t="n"/>
       <c r="C10" s="59" t="n"/>
       <c r="D10" s="59" t="n"/>
       <c r="E10" s="59" t="n"/>
       <c r="F10" s="59" t="n"/>
+      <c r="G10" s="59" t="n"/>
+      <c r="H10" s="59" t="n"/>
+      <c r="I10" s="59" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="J10" s="59" t="n"/>
+      <c r="K10" s="59" t="n"/>
+      <c r="L10" s="59" t="n"/>
+      <c r="M10" s="59" t="n"/>
+      <c r="N10" s="59" t="n"/>
+      <c r="O10" s="59" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="60" t="inlineStr">
@@ -3466,15 +3533,24 @@
           <t>Código</t>
         </is>
       </c>
-      <c r="B11" s="60" t="inlineStr">
-        <is>
-          <t>HD-VENT-001</t>
-        </is>
-      </c>
+      <c r="B11" s="61" t="n"/>
       <c r="C11" s="61" t="n"/>
       <c r="D11" s="61" t="n"/>
       <c r="E11" s="61" t="n"/>
       <c r="F11" s="61" t="n"/>
+      <c r="G11" s="61" t="n"/>
+      <c r="H11" s="61" t="n"/>
+      <c r="I11" s="60" t="inlineStr">
+        <is>
+          <t>HD-VENT-001</t>
+        </is>
+      </c>
+      <c r="J11" s="61" t="n"/>
+      <c r="K11" s="61" t="n"/>
+      <c r="L11" s="61" t="n"/>
+      <c r="M11" s="61" t="n"/>
+      <c r="N11" s="61" t="n"/>
+      <c r="O11" s="61" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="60" t="inlineStr">
@@ -3482,15 +3558,24 @@
           <t>Revisión</t>
         </is>
       </c>
-      <c r="B12" s="60" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="B12" s="61" t="n"/>
       <c r="C12" s="61" t="n"/>
       <c r="D12" s="61" t="n"/>
       <c r="E12" s="61" t="n"/>
       <c r="F12" s="61" t="n"/>
+      <c r="G12" s="61" t="n"/>
+      <c r="H12" s="61" t="n"/>
+      <c r="I12" s="60" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J12" s="61" t="n"/>
+      <c r="K12" s="61" t="n"/>
+      <c r="L12" s="61" t="n"/>
+      <c r="M12" s="61" t="n"/>
+      <c r="N12" s="61" t="n"/>
+      <c r="O12" s="61" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="60" t="inlineStr">
@@ -3498,15 +3583,24 @@
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B13" s="60" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
-        </is>
-      </c>
+      <c r="B13" s="61" t="n"/>
       <c r="C13" s="61" t="n"/>
       <c r="D13" s="61" t="n"/>
       <c r="E13" s="61" t="n"/>
       <c r="F13" s="61" t="n"/>
+      <c r="G13" s="61" t="n"/>
+      <c r="H13" s="61" t="n"/>
+      <c r="I13" s="60" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J13" s="61" t="n"/>
+      <c r="K13" s="61" t="n"/>
+      <c r="L13" s="61" t="n"/>
+      <c r="M13" s="61" t="n"/>
+      <c r="N13" s="61" t="n"/>
+      <c r="O13" s="61" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="60" t="inlineStr">
@@ -3514,15 +3608,24 @@
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B14" s="60" t="inlineStr">
-        <is>
-          <t>P2437-HV-INF-001 — BRINSA, laboratorio de análisis industrial, Cajicá</t>
-        </is>
-      </c>
+      <c r="B14" s="61" t="n"/>
       <c r="C14" s="61" t="n"/>
       <c r="D14" s="61" t="n"/>
       <c r="E14" s="61" t="n"/>
       <c r="F14" s="61" t="n"/>
+      <c r="G14" s="61" t="n"/>
+      <c r="H14" s="61" t="n"/>
+      <c r="I14" s="60" t="inlineStr">
+        <is>
+          <t>P2437-HV-INF-001 — BRINSA, laboratorio de análisis industrial, Cajicá</t>
+        </is>
+      </c>
+      <c r="J14" s="61" t="n"/>
+      <c r="K14" s="61" t="n"/>
+      <c r="L14" s="61" t="n"/>
+      <c r="M14" s="61" t="n"/>
+      <c r="N14" s="61" t="n"/>
+      <c r="O14" s="61" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="60" t="inlineStr">
@@ -3530,15 +3633,24 @@
           <t>Etiqueta de equipo</t>
         </is>
       </c>
-      <c r="B15" s="60" t="inlineStr">
-        <is>
-          <t>VENT-001 (ventilador de impulsión / presurización)</t>
-        </is>
-      </c>
+      <c r="B15" s="61" t="n"/>
       <c r="C15" s="61" t="n"/>
       <c r="D15" s="61" t="n"/>
       <c r="E15" s="61" t="n"/>
       <c r="F15" s="61" t="n"/>
+      <c r="G15" s="61" t="n"/>
+      <c r="H15" s="61" t="n"/>
+      <c r="I15" s="60" t="inlineStr">
+        <is>
+          <t>VENT-001 (ventilador de impulsión / presurización)</t>
+        </is>
+      </c>
+      <c r="J15" s="61" t="n"/>
+      <c r="K15" s="61" t="n"/>
+      <c r="L15" s="61" t="n"/>
+      <c r="M15" s="61" t="n"/>
+      <c r="N15" s="61" t="n"/>
+      <c r="O15" s="61" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="62" t="inlineStr">
@@ -3556,899 +3668,1336 @@
     </row>
     <row r="20"/>
     <row r="21"/>
-    <row r="22"/>
-    <row r="23">
-      <c r="A23" s="63" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="63" t="inlineStr">
         <is>
           <t>1.2. Ambiente de instalación: exterior o semi-cubierto dentro de planta de hipoclorito de calcio; atmósfera con Cl₂/ClO⁻, polvo de Ca(ClO)₂ y humedad relativa media 84 %. Servicio clasificado como altamente corrosivo.</t>
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25"/>
+    <row r="23"/>
+    <row r="25">
+      <c r="A25" s="62" t="inlineStr">
+        <is>
+          <t>2. Condiciones de sitio</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="64" t="inlineStr">
+        <is>
+          <t>Tabla 1. Condiciones ambientales de diseño (fuentes en informe_investigacion.md §3.1; consulta 2026-07-23).</t>
+        </is>
+      </c>
+    </row>
     <row r="27">
-      <c r="A27" s="62" t="inlineStr">
-        <is>
-          <t>2. Condiciones de sitio</t>
-        </is>
-      </c>
+      <c r="A27" s="59" t="inlineStr">
+        <is>
+          <t>Parámetro</t>
+        </is>
+      </c>
+      <c r="B27" s="59" t="n"/>
+      <c r="C27" s="59" t="n"/>
+      <c r="D27" s="59" t="n"/>
+      <c r="E27" s="59" t="n"/>
+      <c r="F27" s="59" t="n"/>
+      <c r="G27" s="59" t="n"/>
+      <c r="H27" s="59" t="n"/>
+      <c r="I27" s="59" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="J27" s="59" t="n"/>
+      <c r="K27" s="59" t="n"/>
+      <c r="L27" s="59" t="n"/>
+      <c r="M27" s="59" t="n"/>
+      <c r="N27" s="59" t="n"/>
+      <c r="O27" s="59" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="64" t="inlineStr">
-        <is>
-          <t>Tabla 1. Condiciones ambientales de diseño (fuentes en informe_investigacion.md §3.1; consulta 2026-07-23).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29"/>
+      <c r="A28" s="60" t="inlineStr">
+        <is>
+          <t>Altitud</t>
+        </is>
+      </c>
+      <c r="B28" s="61" t="n"/>
+      <c r="C28" s="61" t="n"/>
+      <c r="D28" s="61" t="n"/>
+      <c r="E28" s="61" t="n"/>
+      <c r="F28" s="61" t="n"/>
+      <c r="G28" s="61" t="n"/>
+      <c r="H28" s="61" t="n"/>
+      <c r="I28" s="60" t="inlineStr">
+        <is>
+          <t>2 558 msnm</t>
+        </is>
+      </c>
+      <c r="J28" s="61" t="n"/>
+      <c r="K28" s="61" t="n"/>
+      <c r="L28" s="61" t="n"/>
+      <c r="M28" s="61" t="n"/>
+      <c r="N28" s="61" t="n"/>
+      <c r="O28" s="61" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="60" t="inlineStr">
+        <is>
+          <t>Presión atmosférica</t>
+        </is>
+      </c>
+      <c r="B29" s="61" t="n"/>
+      <c r="C29" s="61" t="n"/>
+      <c r="D29" s="61" t="n"/>
+      <c r="E29" s="61" t="n"/>
+      <c r="F29" s="61" t="n"/>
+      <c r="G29" s="61" t="n"/>
+      <c r="H29" s="61" t="n"/>
+      <c r="I29" s="60" t="inlineStr">
+        <is>
+          <t>74.1 kPa</t>
+        </is>
+      </c>
+      <c r="J29" s="61" t="n"/>
+      <c r="K29" s="61" t="n"/>
+      <c r="L29" s="61" t="n"/>
+      <c r="M29" s="61" t="n"/>
+      <c r="N29" s="61" t="n"/>
+      <c r="O29" s="61" t="n"/>
+    </row>
     <row r="30">
-      <c r="A30" s="59" t="inlineStr">
-        <is>
-          <t>Parámetro</t>
-        </is>
-      </c>
-      <c r="B30" s="59" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-      <c r="C30" s="59" t="n"/>
-      <c r="D30" s="59" t="n"/>
-      <c r="E30" s="59" t="n"/>
-      <c r="F30" s="59" t="n"/>
+      <c r="A30" s="60" t="inlineStr">
+        <is>
+          <t>Temperatura de diseño verano / invierno / media</t>
+        </is>
+      </c>
+      <c r="B30" s="61" t="n"/>
+      <c r="C30" s="61" t="n"/>
+      <c r="D30" s="61" t="n"/>
+      <c r="E30" s="61" t="n"/>
+      <c r="F30" s="61" t="n"/>
+      <c r="G30" s="61" t="n"/>
+      <c r="H30" s="61" t="n"/>
+      <c r="I30" s="60" t="inlineStr">
+        <is>
+          <t>21 °C / 3 °C / 14 °C</t>
+        </is>
+      </c>
+      <c r="J30" s="61" t="n"/>
+      <c r="K30" s="61" t="n"/>
+      <c r="L30" s="61" t="n"/>
+      <c r="M30" s="61" t="n"/>
+      <c r="N30" s="61" t="n"/>
+      <c r="O30" s="61" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="60" t="inlineStr">
         <is>
-          <t>Altitud</t>
-        </is>
-      </c>
-      <c r="B31" s="60" t="inlineStr">
-        <is>
-          <t>2 558 msnm</t>
-        </is>
-      </c>
+          <t>Humedad relativa media anual</t>
+        </is>
+      </c>
+      <c r="B31" s="61" t="n"/>
       <c r="C31" s="61" t="n"/>
       <c r="D31" s="61" t="n"/>
       <c r="E31" s="61" t="n"/>
       <c r="F31" s="61" t="n"/>
+      <c r="G31" s="61" t="n"/>
+      <c r="H31" s="61" t="n"/>
+      <c r="I31" s="60" t="inlineStr">
+        <is>
+          <t>84 %</t>
+        </is>
+      </c>
+      <c r="J31" s="61" t="n"/>
+      <c r="K31" s="61" t="n"/>
+      <c r="L31" s="61" t="n"/>
+      <c r="M31" s="61" t="n"/>
+      <c r="N31" s="61" t="n"/>
+      <c r="O31" s="61" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="60" t="inlineStr">
         <is>
-          <t>Presión atmosférica</t>
-        </is>
-      </c>
-      <c r="B32" s="60" t="inlineStr">
-        <is>
-          <t>74.1 kPa</t>
-        </is>
-      </c>
+          <t>Densidad del aire de diseño</t>
+        </is>
+      </c>
+      <c r="B32" s="61" t="n"/>
       <c r="C32" s="61" t="n"/>
       <c r="D32" s="61" t="n"/>
       <c r="E32" s="61" t="n"/>
       <c r="F32" s="61" t="n"/>
+      <c r="G32" s="61" t="n"/>
+      <c r="H32" s="61" t="n"/>
+      <c r="I32" s="60" t="inlineStr">
+        <is>
+          <t>0.88 kg/m³ a 20 °C (0.87 kg/m³ en condición 0.4 %)</t>
+        </is>
+      </c>
+      <c r="J32" s="61" t="n"/>
+      <c r="K32" s="61" t="n"/>
+      <c r="L32" s="61" t="n"/>
+      <c r="M32" s="61" t="n"/>
+      <c r="N32" s="61" t="n"/>
+      <c r="O32" s="61" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="60" t="inlineStr">
         <is>
-          <t>Temperatura de diseño verano / invierno / media</t>
-        </is>
-      </c>
-      <c r="B33" s="60" t="inlineStr">
-        <is>
-          <t>21 °C / 3 °C / 14 °C</t>
-        </is>
-      </c>
+          <t>Factor de densidad k (vs. catálogo 1.2 kg/m³)</t>
+        </is>
+      </c>
+      <c r="B33" s="61" t="n"/>
       <c r="C33" s="61" t="n"/>
       <c r="D33" s="61" t="n"/>
       <c r="E33" s="61" t="n"/>
       <c r="F33" s="61" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="60" t="inlineStr">
-        <is>
-          <t>Humedad relativa media anual</t>
-        </is>
-      </c>
-      <c r="B34" s="60" t="inlineStr">
-        <is>
-          <t>84 %</t>
-        </is>
-      </c>
-      <c r="C34" s="61" t="n"/>
-      <c r="D34" s="61" t="n"/>
-      <c r="E34" s="61" t="n"/>
-      <c r="F34" s="61" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="60" t="inlineStr">
-        <is>
-          <t>Densidad del aire de diseño</t>
-        </is>
-      </c>
-      <c r="B35" s="60" t="inlineStr">
-        <is>
-          <t>0.88 kg/m³ a 20 °C (0.87 kg/m³ en condición 0.4 %)</t>
-        </is>
-      </c>
-      <c r="C35" s="61" t="n"/>
-      <c r="D35" s="61" t="n"/>
-      <c r="E35" s="61" t="n"/>
-      <c r="F35" s="61" t="n"/>
+      <c r="G33" s="61" t="n"/>
+      <c r="H33" s="61" t="n"/>
+      <c r="I33" s="60" t="inlineStr">
+        <is>
+          <t>0.733</t>
+        </is>
+      </c>
+      <c r="J33" s="61" t="n"/>
+      <c r="K33" s="61" t="n"/>
+      <c r="L33" s="61" t="n"/>
+      <c r="M33" s="61" t="n"/>
+      <c r="N33" s="61" t="n"/>
+      <c r="O33" s="61" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="60" t="inlineStr">
-        <is>
-          <t>Factor de densidad k (vs. catálogo 1.2 kg/m³)</t>
-        </is>
-      </c>
-      <c r="B36" s="60" t="inlineStr">
-        <is>
-          <t>0.733</t>
-        </is>
-      </c>
-      <c r="C36" s="61" t="n"/>
-      <c r="D36" s="61" t="n"/>
-      <c r="E36" s="61" t="n"/>
-      <c r="F36" s="61" t="n"/>
+      <c r="A36" s="62" t="inlineStr">
+        <is>
+          <t>3. Punto de trabajo</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="64" t="inlineStr">
+        <is>
+          <t>Tabla 2. Punto de trabajo en el sitio y punto equivalente de selección en catálogo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="59" t="inlineStr">
+        <is>
+          <t>Magnitud</t>
+        </is>
+      </c>
+      <c r="B38" s="59" t="n"/>
+      <c r="C38" s="59" t="n"/>
+      <c r="D38" s="59" t="n"/>
+      <c r="E38" s="59" t="n"/>
+      <c r="F38" s="59" t="inlineStr">
+        <is>
+          <t>En el sitio (ρ = 0.88 kg/m³)</t>
+        </is>
+      </c>
+      <c r="G38" s="59" t="n"/>
+      <c r="H38" s="59" t="n"/>
+      <c r="I38" s="59" t="n"/>
+      <c r="J38" s="59" t="n"/>
+      <c r="K38" s="59" t="inlineStr">
+        <is>
+          <t>Equivalente catálogo (ρ = 1.2 kg/m³)</t>
+        </is>
+      </c>
+      <c r="L38" s="59" t="n"/>
+      <c r="M38" s="59" t="n"/>
+      <c r="N38" s="59" t="n"/>
+      <c r="O38" s="59" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="62" t="inlineStr">
-        <is>
-          <t>3. Punto de trabajo</t>
-        </is>
-      </c>
+      <c r="A39" s="60" t="inlineStr">
+        <is>
+          <t>Caudal</t>
+        </is>
+      </c>
+      <c r="B39" s="61" t="n"/>
+      <c r="C39" s="61" t="n"/>
+      <c r="D39" s="61" t="n"/>
+      <c r="E39" s="61" t="n"/>
+      <c r="F39" s="60" t="inlineStr">
+        <is>
+          <t>3 840 m³/h = 64 m³/min = 1.0667 m³/s = 2 260 CFM</t>
+        </is>
+      </c>
+      <c r="G39" s="61" t="n"/>
+      <c r="H39" s="61" t="n"/>
+      <c r="I39" s="61" t="n"/>
+      <c r="J39" s="61" t="n"/>
+      <c r="K39" s="60" t="inlineStr">
+        <is>
+          <t>Sin cambio (máquina de volumen constante)</t>
+        </is>
+      </c>
+      <c r="L39" s="61" t="n"/>
+      <c r="M39" s="61" t="n"/>
+      <c r="N39" s="61" t="n"/>
+      <c r="O39" s="61" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="64" t="inlineStr">
-        <is>
-          <t>Tabla 2. Punto de trabajo en el sitio y punto equivalente de selección en catálogo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41"/>
+      <c r="A40" s="60" t="inlineStr">
+        <is>
+          <t>ΔP total, escenario de diseño (filtro cargado)</t>
+        </is>
+      </c>
+      <c r="B40" s="61" t="n"/>
+      <c r="C40" s="61" t="n"/>
+      <c r="D40" s="61" t="n"/>
+      <c r="E40" s="61" t="n"/>
+      <c r="F40" s="60" t="inlineStr">
+        <is>
+          <t>190 Pa</t>
+        </is>
+      </c>
+      <c r="G40" s="61" t="n"/>
+      <c r="H40" s="61" t="n"/>
+      <c r="I40" s="61" t="n"/>
+      <c r="J40" s="61" t="n"/>
+      <c r="K40" s="60" t="inlineStr">
+        <is>
+          <t>260 Pa</t>
+        </is>
+      </c>
+      <c r="L40" s="61" t="n"/>
+      <c r="M40" s="61" t="n"/>
+      <c r="N40" s="61" t="n"/>
+      <c r="O40" s="61" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="60" t="inlineStr">
+        <is>
+          <t>ΔP total, escenario filtro limpio</t>
+        </is>
+      </c>
+      <c r="B41" s="61" t="n"/>
+      <c r="C41" s="61" t="n"/>
+      <c r="D41" s="61" t="n"/>
+      <c r="E41" s="61" t="n"/>
+      <c r="F41" s="60" t="inlineStr">
+        <is>
+          <t>95 Pa</t>
+        </is>
+      </c>
+      <c r="G41" s="61" t="n"/>
+      <c r="H41" s="61" t="n"/>
+      <c r="I41" s="61" t="n"/>
+      <c r="J41" s="61" t="n"/>
+      <c r="K41" s="60" t="inlineStr">
+        <is>
+          <t>130 Pa</t>
+        </is>
+      </c>
+      <c r="L41" s="61" t="n"/>
+      <c r="M41" s="61" t="n"/>
+      <c r="N41" s="61" t="n"/>
+      <c r="O41" s="61" t="n"/>
+    </row>
     <row r="42">
-      <c r="A42" s="59" t="inlineStr">
-        <is>
-          <t>Magnitud</t>
-        </is>
-      </c>
-      <c r="B42" s="59" t="inlineStr">
-        <is>
-          <t>En el sitio (ρ = 0.88 kg/m³)</t>
-        </is>
-      </c>
-      <c r="C42" s="59" t="inlineStr">
-        <is>
-          <t>Equivalente catálogo (ρ = 1.2 kg/m³)</t>
-        </is>
-      </c>
-      <c r="D42" s="59" t="n"/>
-      <c r="E42" s="59" t="n"/>
-      <c r="F42" s="59" t="n"/>
+      <c r="A42" s="60" t="inlineStr">
+        <is>
+          <t>Composición ΔP diseño</t>
+        </is>
+      </c>
+      <c r="B42" s="61" t="n"/>
+      <c r="C42" s="61" t="n"/>
+      <c r="D42" s="61" t="n"/>
+      <c r="E42" s="61" t="n"/>
+      <c r="F42" s="60" t="inlineStr">
+        <is>
+          <t>Filtro 154 Pa + presurización 25 Pa + rejillas 11 Pa</t>
+        </is>
+      </c>
+      <c r="G42" s="61" t="n"/>
+      <c r="H42" s="61" t="n"/>
+      <c r="I42" s="61" t="n"/>
+      <c r="J42" s="61" t="n"/>
+      <c r="K42" s="60" t="inlineStr">
+        <is>
+          <t>Filtro 210 Pa + 34 Pa + 15 Pa</t>
+        </is>
+      </c>
+      <c r="L42" s="61" t="n"/>
+      <c r="M42" s="61" t="n"/>
+      <c r="N42" s="61" t="n"/>
+      <c r="O42" s="61" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="60" t="inlineStr">
         <is>
-          <t>Caudal</t>
-        </is>
-      </c>
-      <c r="B43" s="60" t="inlineStr">
-        <is>
-          <t>3 840 m³/h = 64 m³/min = 1.0667 m³/s = 2 260 CFM</t>
-        </is>
-      </c>
-      <c r="C43" s="60" t="inlineStr">
-        <is>
-          <t>Sin cambio (máquina de volumen constante)</t>
-        </is>
-      </c>
+          <t>Velocidad de inyección</t>
+        </is>
+      </c>
+      <c r="B43" s="61" t="n"/>
+      <c r="C43" s="61" t="n"/>
       <c r="D43" s="61" t="n"/>
       <c r="E43" s="61" t="n"/>
-      <c r="F43" s="61" t="n"/>
+      <c r="F43" s="60" t="inlineStr">
+        <is>
+          <t>8 m/s (presión dinámica 28 Pa en el sitio)</t>
+        </is>
+      </c>
+      <c r="G43" s="61" t="n"/>
+      <c r="H43" s="61" t="n"/>
+      <c r="I43" s="61" t="n"/>
+      <c r="J43" s="61" t="n"/>
+      <c r="K43" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L43" s="61" t="n"/>
+      <c r="M43" s="61" t="n"/>
+      <c r="N43" s="61" t="n"/>
+      <c r="O43" s="61" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="60" t="inlineStr">
         <is>
-          <t>ΔP total, escenario de diseño (filtro cargado)</t>
-        </is>
-      </c>
-      <c r="B44" s="60" t="inlineStr">
-        <is>
-          <t>190 Pa</t>
-        </is>
-      </c>
-      <c r="C44" s="60" t="inlineStr">
-        <is>
-          <t>260 Pa</t>
-        </is>
-      </c>
+          <t>Potencia teórica al freno (η = 0.60)</t>
+        </is>
+      </c>
+      <c r="B44" s="61" t="n"/>
+      <c r="C44" s="61" t="n"/>
       <c r="D44" s="61" t="n"/>
       <c r="E44" s="61" t="n"/>
-      <c r="F44" s="61" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="60" t="inlineStr">
-        <is>
-          <t>ΔP total, escenario filtro limpio</t>
-        </is>
-      </c>
-      <c r="B45" s="60" t="inlineStr">
-        <is>
-          <t>95 Pa</t>
-        </is>
-      </c>
-      <c r="C45" s="60" t="inlineStr">
-        <is>
-          <t>130 Pa</t>
-        </is>
-      </c>
-      <c r="D45" s="61" t="n"/>
-      <c r="E45" s="61" t="n"/>
-      <c r="F45" s="61" t="n"/>
+      <c r="F44" s="60" t="inlineStr">
+        <is>
+          <t>0.338 kW = 0.45 HP</t>
+        </is>
+      </c>
+      <c r="G44" s="61" t="n"/>
+      <c r="H44" s="61" t="n"/>
+      <c r="I44" s="61" t="n"/>
+      <c r="J44" s="61" t="n"/>
+      <c r="K44" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L44" s="61" t="n"/>
+      <c r="M44" s="61" t="n"/>
+      <c r="N44" s="61" t="n"/>
+      <c r="O44" s="61" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="60" t="inlineStr">
-        <is>
-          <t>Composición ΔP diseño</t>
-        </is>
-      </c>
-      <c r="B46" s="60" t="inlineStr">
-        <is>
-          <t>Filtro 154 Pa + presurización 25 Pa + rejillas 11 Pa</t>
-        </is>
-      </c>
-      <c r="C46" s="60" t="inlineStr">
-        <is>
-          <t>Filtro 210 Pa + 34 Pa + 15 Pa</t>
-        </is>
-      </c>
-      <c r="D46" s="61" t="n"/>
-      <c r="E46" s="61" t="n"/>
-      <c r="F46" s="61" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="60" t="inlineStr">
-        <is>
-          <t>Velocidad de inyección</t>
-        </is>
-      </c>
-      <c r="B47" s="60" t="inlineStr">
-        <is>
-          <t>8 m/s (presión dinámica 28 Pa en el sitio)</t>
-        </is>
-      </c>
-      <c r="C47" s="60" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D47" s="61" t="n"/>
-      <c r="E47" s="61" t="n"/>
-      <c r="F47" s="61" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="60" t="inlineStr">
-        <is>
-          <t>Potencia teórica al freno (η = 0.60)</t>
-        </is>
-      </c>
-      <c r="B48" s="60" t="inlineStr">
-        <is>
-          <t>0.338 kW = 0.45 HP</t>
-        </is>
-      </c>
-      <c r="C48" s="60" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D48" s="61" t="n"/>
-      <c r="E48" s="61" t="n"/>
-      <c r="F48" s="61" t="n"/>
-    </row>
+      <c r="A46" s="63" t="inlineStr">
+        <is>
+          <t>3.1. La selección se efectúa sobre catálogo a densidad estándar en el punto 3 840 m³/h @ 260 Pa, aplicando las leyes de los ventiladores (P ∝ ρ, potencia ∝ ρ, Q constante) según Twin City Fan FE-1600 (http://eu.tcf.com/wp-content/uploads/sites/4/2018/06/Temperature-Altitude-Effects-on-Fans-FE-1600-1.pdf) (consulta 2026-07-23). Tamaño y RPM exactos: por confirmar con proveedor mediante su software de selección.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
     <row r="50">
       <c r="A50" s="63" t="inlineStr">
         <is>
-          <t>3.1. La selección se efectúa sobre catálogo a densidad estándar en el punto 3 840 m³/h @ 260 Pa, aplicando las leyes de los ventiladores (P ∝ ρ, potencia ∝ ρ, Q constante) según Twin City Fan FE-1600 (http://eu.tcf.com/wp-content/uploads/sites/4/2018/06/Temperature-Altitude-Effects-on-Fans-FE-1600-1.pdf) (consulta 2026-07-23). Tamaño y RPM exactos: por confirmar con proveedor mediante su software de selección.</t>
+          <t>3.2. El ventilador seleccionado entregará en el sitio el mismo caudal a las mismas RPM, con presión y potencia reducidas en el factor 0.733; el margen sobre la potencia de eje (motor 1.0 HP vs. 0.45 HP teóricos) absorbe el derateo por altitud de NEMA MG-1 (≈9 % a 2 558 msnm) y el factor de servicio.</t>
         </is>
       </c>
     </row>
     <row r="51"/>
     <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
+    <row r="54">
+      <c r="A54" s="62" t="inlineStr">
+        <is>
+          <t>4. Tipo y materiales de construcción</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="64" t="inlineStr">
+        <is>
+          <t>Tabla 3. Requisitos de construcción.</t>
+        </is>
+      </c>
+    </row>
     <row r="56">
-      <c r="A56" s="63" t="inlineStr">
-        <is>
-          <t>3.2. El ventilador seleccionado entregará en el sitio el mismo caudal a las mismas RPM, con presión y potencia reducidas en el factor 0.733; el margen sobre la potencia de eje (motor 1.0 HP vs. 0.45 HP teóricos) absorbe el derateo por altitud de NEMA MG-1 (≈9 % a 2 558 msnm) y el factor de servicio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
+      <c r="A56" s="59" t="inlineStr">
+        <is>
+          <t>Componente</t>
+        </is>
+      </c>
+      <c r="B56" s="59" t="n"/>
+      <c r="C56" s="59" t="n"/>
+      <c r="D56" s="59" t="n"/>
+      <c r="E56" s="59" t="n"/>
+      <c r="F56" s="59" t="n"/>
+      <c r="G56" s="59" t="n"/>
+      <c r="H56" s="59" t="n"/>
+      <c r="I56" s="59" t="inlineStr">
+        <is>
+          <t>Especificación</t>
+        </is>
+      </c>
+      <c r="J56" s="59" t="n"/>
+      <c r="K56" s="59" t="n"/>
+      <c r="L56" s="59" t="n"/>
+      <c r="M56" s="59" t="n"/>
+      <c r="N56" s="59" t="n"/>
+      <c r="O56" s="59" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="60" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="B57" s="61" t="n"/>
+      <c r="C57" s="61" t="n"/>
+      <c r="D57" s="61" t="n"/>
+      <c r="E57" s="61" t="n"/>
+      <c r="F57" s="61" t="n"/>
+      <c r="G57" s="61" t="n"/>
+      <c r="H57" s="61" t="n"/>
+      <c r="I57" s="60" t="inlineStr">
+        <is>
+          <t>Centrífugo, álabes curvados hacia atrás, simple aspiración, transmisión directa o por bandas (dato típico según línea seleccionada)</t>
+        </is>
+      </c>
+      <c r="J57" s="61" t="n"/>
+      <c r="K57" s="61" t="n"/>
+      <c r="L57" s="61" t="n"/>
+      <c r="M57" s="61" t="n"/>
+      <c r="N57" s="61" t="n"/>
+      <c r="O57" s="61" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="60" t="inlineStr">
+        <is>
+          <t>Carcasa y rueda</t>
+        </is>
+      </c>
+      <c r="B58" s="61" t="n"/>
+      <c r="C58" s="61" t="n"/>
+      <c r="D58" s="61" t="n"/>
+      <c r="E58" s="61" t="n"/>
+      <c r="F58" s="61" t="n"/>
+      <c r="G58" s="61" t="n"/>
+      <c r="H58" s="61" t="n"/>
+      <c r="I58" s="60" t="inlineStr">
+        <is>
+          <t>PRFV con resina viniléster, laminado según ASTM C582/D4167 (primera opción) o polipropileno (alternativa); velo superficial para oxidantes fuertes donde el fabricante lo ofrezca</t>
+        </is>
+      </c>
+      <c r="J58" s="61" t="n"/>
+      <c r="K58" s="61" t="n"/>
+      <c r="L58" s="61" t="n"/>
+      <c r="M58" s="61" t="n"/>
+      <c r="N58" s="61" t="n"/>
+      <c r="O58" s="61" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="60" t="inlineStr">
+        <is>
+          <t>Elementos metálicos en la corriente</t>
+        </is>
+      </c>
+      <c r="B59" s="61" t="n"/>
+      <c r="C59" s="61" t="n"/>
+      <c r="D59" s="61" t="n"/>
+      <c r="E59" s="61" t="n"/>
+      <c r="F59" s="61" t="n"/>
+      <c r="G59" s="61" t="n"/>
+      <c r="H59" s="61" t="n"/>
+      <c r="I59" s="60" t="inlineStr">
+        <is>
+          <t>Ninguno (motor fuera de la corriente de aire)</t>
+        </is>
+      </c>
+      <c r="J59" s="61" t="n"/>
+      <c r="K59" s="61" t="n"/>
+      <c r="L59" s="61" t="n"/>
+      <c r="M59" s="61" t="n"/>
+      <c r="N59" s="61" t="n"/>
+      <c r="O59" s="61" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="60" t="inlineStr">
+        <is>
+          <t>Eje y buje</t>
+        </is>
+      </c>
+      <c r="B60" s="61" t="n"/>
+      <c r="C60" s="61" t="n"/>
+      <c r="D60" s="61" t="n"/>
+      <c r="E60" s="61" t="n"/>
+      <c r="F60" s="61" t="n"/>
+      <c r="G60" s="61" t="n"/>
+      <c r="H60" s="61" t="n"/>
+      <c r="I60" s="60" t="inlineStr">
+        <is>
+          <t>Encapsulados/protegidos contra la atmósfera clorada</t>
+        </is>
+      </c>
+      <c r="J60" s="61" t="n"/>
+      <c r="K60" s="61" t="n"/>
+      <c r="L60" s="61" t="n"/>
+      <c r="M60" s="61" t="n"/>
+      <c r="N60" s="61" t="n"/>
+      <c r="O60" s="61" t="n"/>
+    </row>
     <row r="61">
-      <c r="A61" s="62" t="inlineStr">
-        <is>
-          <t>4. Tipo y materiales de construcción</t>
-        </is>
-      </c>
+      <c r="A61" s="60" t="inlineStr">
+        <is>
+          <t>Construcción contra chispa</t>
+        </is>
+      </c>
+      <c r="B61" s="61" t="n"/>
+      <c r="C61" s="61" t="n"/>
+      <c r="D61" s="61" t="n"/>
+      <c r="E61" s="61" t="n"/>
+      <c r="F61" s="61" t="n"/>
+      <c r="G61" s="61" t="n"/>
+      <c r="H61" s="61" t="n"/>
+      <c r="I61" s="60" t="inlineStr">
+        <is>
+          <t>AMCA 99 Spark A (dato típico de especificación para PRFV)</t>
+        </is>
+      </c>
+      <c r="J61" s="61" t="n"/>
+      <c r="K61" s="61" t="n"/>
+      <c r="L61" s="61" t="n"/>
+      <c r="M61" s="61" t="n"/>
+      <c r="N61" s="61" t="n"/>
+      <c r="O61" s="61" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="64" t="inlineStr">
-        <is>
-          <t>Tabla 3. Requisitos de construcción.</t>
-        </is>
-      </c>
+      <c r="A62" s="60" t="inlineStr">
+        <is>
+          <t>Certificación de desempeño</t>
+        </is>
+      </c>
+      <c r="B62" s="61" t="n"/>
+      <c r="C62" s="61" t="n"/>
+      <c r="D62" s="61" t="n"/>
+      <c r="E62" s="61" t="n"/>
+      <c r="F62" s="61" t="n"/>
+      <c r="G62" s="61" t="n"/>
+      <c r="H62" s="61" t="n"/>
+      <c r="I62" s="60" t="inlineStr">
+        <is>
+          <t>AMCA 210/211 (sello AMCA exigible)</t>
+        </is>
+      </c>
+      <c r="J62" s="61" t="n"/>
+      <c r="K62" s="61" t="n"/>
+      <c r="L62" s="61" t="n"/>
+      <c r="M62" s="61" t="n"/>
+      <c r="N62" s="61" t="n"/>
+      <c r="O62" s="61" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="59" t="inlineStr">
-        <is>
-          <t>Componente</t>
-        </is>
-      </c>
-      <c r="B63" s="59" t="inlineStr">
-        <is>
-          <t>Especificación</t>
-        </is>
-      </c>
-      <c r="C63" s="59" t="n"/>
-      <c r="D63" s="59" t="n"/>
-      <c r="E63" s="59" t="n"/>
-      <c r="F63" s="59" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="60" t="inlineStr">
-        <is>
-          <t>Tipo</t>
-        </is>
-      </c>
-      <c r="B64" s="60" t="inlineStr">
-        <is>
-          <t>Centrífugo, álabes curvados hacia atrás, simple aspiración, transmisión directa o por bandas (dato típico según línea seleccionada)</t>
-        </is>
-      </c>
-      <c r="C64" s="61" t="n"/>
-      <c r="D64" s="61" t="n"/>
-      <c r="E64" s="61" t="n"/>
-      <c r="F64" s="61" t="n"/>
+      <c r="A63" s="60" t="inlineStr">
+        <is>
+          <t>Descartado</t>
+        </is>
+      </c>
+      <c r="B63" s="61" t="n"/>
+      <c r="C63" s="61" t="n"/>
+      <c r="D63" s="61" t="n"/>
+      <c r="E63" s="61" t="n"/>
+      <c r="F63" s="61" t="n"/>
+      <c r="G63" s="61" t="n"/>
+      <c r="H63" s="61" t="n"/>
+      <c r="I63" s="60" t="inlineStr">
+        <is>
+          <t>Axial PRFV (presión insuficiente con MERV 13-14); acero inoxidable en la corriente (picadura por cloruros); acero galvanizado</t>
+        </is>
+      </c>
+      <c r="J63" s="61" t="n"/>
+      <c r="K63" s="61" t="n"/>
+      <c r="L63" s="61" t="n"/>
+      <c r="M63" s="61" t="n"/>
+      <c r="N63" s="61" t="n"/>
+      <c r="O63" s="61" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="60" t="inlineStr">
-        <is>
-          <t>Carcasa y rueda</t>
-        </is>
-      </c>
-      <c r="B65" s="60" t="inlineStr">
-        <is>
-          <t>PRFV con resina viniléster, laminado según ASTM C582/D4167 (primera opción) o polipropileno (alternativa); velo superficial para oxidantes fuertes donde el fabricante lo ofrezca</t>
-        </is>
-      </c>
-      <c r="C65" s="61" t="n"/>
-      <c r="D65" s="61" t="n"/>
-      <c r="E65" s="61" t="n"/>
-      <c r="F65" s="61" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="60" t="inlineStr">
-        <is>
-          <t>Elementos metálicos en la corriente</t>
-        </is>
-      </c>
-      <c r="B66" s="60" t="inlineStr">
-        <is>
-          <t>Ninguno (motor fuera de la corriente de aire)</t>
-        </is>
-      </c>
-      <c r="C66" s="61" t="n"/>
-      <c r="D66" s="61" t="n"/>
-      <c r="E66" s="61" t="n"/>
-      <c r="F66" s="61" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="60" t="inlineStr">
-        <is>
-          <t>Eje y buje</t>
-        </is>
-      </c>
-      <c r="B67" s="60" t="inlineStr">
-        <is>
-          <t>Encapsulados/protegidos contra la atmósfera clorada</t>
-        </is>
-      </c>
-      <c r="C67" s="61" t="n"/>
-      <c r="D67" s="61" t="n"/>
-      <c r="E67" s="61" t="n"/>
-      <c r="F67" s="61" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="60" t="inlineStr">
-        <is>
-          <t>Construcción contra chispa</t>
-        </is>
-      </c>
-      <c r="B68" s="60" t="inlineStr">
-        <is>
-          <t>AMCA 99 Spark A (dato típico de especificación para PRFV)</t>
-        </is>
-      </c>
-      <c r="C68" s="61" t="n"/>
-      <c r="D68" s="61" t="n"/>
-      <c r="E68" s="61" t="n"/>
-      <c r="F68" s="61" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="60" t="inlineStr">
-        <is>
-          <t>Certificación de desempeño</t>
-        </is>
-      </c>
-      <c r="B69" s="60" t="inlineStr">
-        <is>
-          <t>AMCA 210/211 (sello AMCA exigible)</t>
-        </is>
-      </c>
-      <c r="C69" s="61" t="n"/>
-      <c r="D69" s="61" t="n"/>
-      <c r="E69" s="61" t="n"/>
-      <c r="F69" s="61" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="60" t="inlineStr">
-        <is>
-          <t>Descartado</t>
-        </is>
-      </c>
-      <c r="B70" s="60" t="inlineStr">
-        <is>
-          <t>Axial PRFV (presión insuficiente con MERV 13-14); acero inoxidable en la corriente (picadura por cloruros); acero galvanizado</t>
-        </is>
-      </c>
-      <c r="C70" s="61" t="n"/>
-      <c r="D70" s="61" t="n"/>
-      <c r="E70" s="61" t="n"/>
-      <c r="F70" s="61" t="n"/>
+      <c r="A65" s="65" t="inlineStr">
+        <is>
+          <t>Justificación de materiales: las resinas viniléster tipo Derakane se especifican expresamente para cloro e hipoclorito (INEOS — Derakane Resin Selection Guide (http://www.ineos.com/globalassets/ineos-group/businesses/ineos-composites/markets/corrosion/derakane-resin-selection-guide.pdf), consulta 2026-07-23); el polipropileno ofrece alta resistencia a cloruros e hipoclorito a temperatura ambiente (Plastec (https://www.plastecventilation.com/collections/plastec-series), consulta 2026-07-23).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="71">
+      <c r="A71" s="62" t="inlineStr">
+        <is>
+          <t>5. Motor</t>
+        </is>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="63" t="inlineStr">
-        <is>
-          <t>Justificación de materiales: las resinas viniléster tipo Derakane se especifican expresamente para cloro e hipoclorito (INEOS — Derakane Resin Selection Guide (http://www.ineos.com/globalassets/ineos-group/businesses/ineos-composites/markets/corrosion/derakane-resin-selection-guide.pdf), consulta 2026-07-23); el polipropileno ofrece alta resistencia a cloruros e hipoclorito a temperatura ambiente (Plastec (https://www.plastecventilation.com/collections/plastec-series), consulta 2026-07-23).</t>
-        </is>
-      </c>
-    </row>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
+      <c r="A72" s="64" t="inlineStr">
+        <is>
+          <t>Tabla 4. Especificación del motor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="59" t="inlineStr">
+        <is>
+          <t>Parámetro</t>
+        </is>
+      </c>
+      <c r="B73" s="59" t="n"/>
+      <c r="C73" s="59" t="n"/>
+      <c r="D73" s="59" t="n"/>
+      <c r="E73" s="59" t="n"/>
+      <c r="F73" s="59" t="n"/>
+      <c r="G73" s="59" t="n"/>
+      <c r="H73" s="59" t="n"/>
+      <c r="I73" s="59" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="J73" s="59" t="n"/>
+      <c r="K73" s="59" t="n"/>
+      <c r="L73" s="59" t="n"/>
+      <c r="M73" s="59" t="n"/>
+      <c r="N73" s="59" t="n"/>
+      <c r="O73" s="59" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="60" t="inlineStr">
+        <is>
+          <t>Potencia instalada</t>
+        </is>
+      </c>
+      <c r="B74" s="61" t="n"/>
+      <c r="C74" s="61" t="n"/>
+      <c r="D74" s="61" t="n"/>
+      <c r="E74" s="61" t="n"/>
+      <c r="F74" s="61" t="n"/>
+      <c r="G74" s="61" t="n"/>
+      <c r="H74" s="61" t="n"/>
+      <c r="I74" s="60" t="inlineStr">
+        <is>
+          <t>1.0 HP</t>
+        </is>
+      </c>
+      <c r="J74" s="61" t="n"/>
+      <c r="K74" s="61" t="n"/>
+      <c r="L74" s="61" t="n"/>
+      <c r="M74" s="61" t="n"/>
+      <c r="N74" s="61" t="n"/>
+      <c r="O74" s="61" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="60" t="inlineStr">
+        <is>
+          <t>Ejecución</t>
+        </is>
+      </c>
+      <c r="B75" s="61" t="n"/>
+      <c r="C75" s="61" t="n"/>
+      <c r="D75" s="61" t="n"/>
+      <c r="E75" s="61" t="n"/>
+      <c r="F75" s="61" t="n"/>
+      <c r="G75" s="61" t="n"/>
+      <c r="H75" s="61" t="n"/>
+      <c r="I75" s="60" t="inlineStr">
+        <is>
+          <t>TEFC, severe duty, pintura epóxica, protección interna anticorrosiva, sellos de eje en ambos extremos (referencia IEEE 841 o equivalente)</t>
+        </is>
+      </c>
+      <c r="J75" s="61" t="n"/>
+      <c r="K75" s="61" t="n"/>
+      <c r="L75" s="61" t="n"/>
+      <c r="M75" s="61" t="n"/>
+      <c r="N75" s="61" t="n"/>
+      <c r="O75" s="61" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="60" t="inlineStr">
+        <is>
+          <t>Velocidad</t>
+        </is>
+      </c>
+      <c r="B76" s="61" t="n"/>
+      <c r="C76" s="61" t="n"/>
+      <c r="D76" s="61" t="n"/>
+      <c r="E76" s="61" t="n"/>
+      <c r="F76" s="61" t="n"/>
+      <c r="G76" s="61" t="n"/>
+      <c r="H76" s="61" t="n"/>
+      <c r="I76" s="60" t="inlineStr">
+        <is>
+          <t>1 800 RPM (4 polos, 60 Hz) — dato típico</t>
+        </is>
+      </c>
+      <c r="J76" s="61" t="n"/>
+      <c r="K76" s="61" t="n"/>
+      <c r="L76" s="61" t="n"/>
+      <c r="M76" s="61" t="n"/>
+      <c r="N76" s="61" t="n"/>
+      <c r="O76" s="61" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="60" t="inlineStr">
+        <is>
+          <t>Aislamiento / protección</t>
+        </is>
+      </c>
+      <c r="B77" s="61" t="n"/>
+      <c r="C77" s="61" t="n"/>
+      <c r="D77" s="61" t="n"/>
+      <c r="E77" s="61" t="n"/>
+      <c r="F77" s="61" t="n"/>
+      <c r="G77" s="61" t="n"/>
+      <c r="H77" s="61" t="n"/>
+      <c r="I77" s="60" t="inlineStr">
+        <is>
+          <t>Clase F / IP55 mínimo (IP56 preferible)</t>
+        </is>
+      </c>
+      <c r="J77" s="61" t="n"/>
+      <c r="K77" s="61" t="n"/>
+      <c r="L77" s="61" t="n"/>
+      <c r="M77" s="61" t="n"/>
+      <c r="N77" s="61" t="n"/>
+      <c r="O77" s="61" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="60" t="inlineStr">
+        <is>
+          <t>Tensión / fases / frecuencia</t>
+        </is>
+      </c>
+      <c r="B78" s="61" t="n"/>
+      <c r="C78" s="61" t="n"/>
+      <c r="D78" s="61" t="n"/>
+      <c r="E78" s="61" t="n"/>
+      <c r="F78" s="61" t="n"/>
+      <c r="G78" s="61" t="n"/>
+      <c r="H78" s="61" t="n"/>
+      <c r="I78" s="60" t="inlineStr">
+        <is>
+          <t>440 V, 3φ, 60 Hz (confirmado por el cliente, 2026-07-23)</t>
+        </is>
+      </c>
+      <c r="J78" s="61" t="n"/>
+      <c r="K78" s="61" t="n"/>
+      <c r="L78" s="61" t="n"/>
+      <c r="M78" s="61" t="n"/>
+      <c r="N78" s="61" t="n"/>
+      <c r="O78" s="61" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="60" t="inlineStr">
+        <is>
+          <t>Derateo por altitud</t>
+        </is>
+      </c>
+      <c r="B79" s="61" t="n"/>
+      <c r="C79" s="61" t="n"/>
+      <c r="D79" s="61" t="n"/>
+      <c r="E79" s="61" t="n"/>
+      <c r="F79" s="61" t="n"/>
+      <c r="G79" s="61" t="n"/>
+      <c r="H79" s="61" t="n"/>
+      <c r="I79" s="60" t="inlineStr">
+        <is>
+          <t>≈9 % (NEMA MG-1); absorbido por el margen de selección (§3.2)</t>
+        </is>
+      </c>
+      <c r="J79" s="61" t="n"/>
+      <c r="K79" s="61" t="n"/>
+      <c r="L79" s="61" t="n"/>
+      <c r="M79" s="61" t="n"/>
+      <c r="N79" s="61" t="n"/>
+      <c r="O79" s="61" t="n"/>
+    </row>
     <row r="80">
-      <c r="A80" s="62" t="inlineStr">
-        <is>
-          <t>5. Motor</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="64" t="inlineStr">
-        <is>
-          <t>Tabla 4. Especificación del motor.</t>
-        </is>
-      </c>
+      <c r="A80" s="60" t="inlineStr">
+        <is>
+          <t>Accesorios</t>
+        </is>
+      </c>
+      <c r="B80" s="61" t="n"/>
+      <c r="C80" s="61" t="n"/>
+      <c r="D80" s="61" t="n"/>
+      <c r="E80" s="61" t="n"/>
+      <c r="F80" s="61" t="n"/>
+      <c r="G80" s="61" t="n"/>
+      <c r="H80" s="61" t="n"/>
+      <c r="I80" s="60" t="inlineStr">
+        <is>
+          <t>Calentador anticondensación si hay paradas largas (dato típico de buena práctica); caja de conexiones sellada, prensaestopas niquelados</t>
+        </is>
+      </c>
+      <c r="J80" s="61" t="n"/>
+      <c r="K80" s="61" t="n"/>
+      <c r="L80" s="61" t="n"/>
+      <c r="M80" s="61" t="n"/>
+      <c r="N80" s="61" t="n"/>
+      <c r="O80" s="61" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="59" t="inlineStr">
-        <is>
-          <t>Parámetro</t>
-        </is>
-      </c>
-      <c r="B82" s="59" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-      <c r="C82" s="59" t="n"/>
-      <c r="D82" s="59" t="n"/>
-      <c r="E82" s="59" t="n"/>
-      <c r="F82" s="59" t="n"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="60" t="inlineStr">
-        <is>
-          <t>Potencia instalada</t>
-        </is>
-      </c>
-      <c r="B83" s="60" t="inlineStr">
-        <is>
-          <t>1.0 HP</t>
-        </is>
-      </c>
-      <c r="C83" s="61" t="n"/>
-      <c r="D83" s="61" t="n"/>
-      <c r="E83" s="61" t="n"/>
-      <c r="F83" s="61" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="60" t="inlineStr">
-        <is>
-          <t>Ejecución</t>
-        </is>
-      </c>
-      <c r="B84" s="60" t="inlineStr">
-        <is>
-          <t>TEFC, severe duty, pintura epóxica, protección interna anticorrosiva, sellos de eje en ambos extremos (referencia IEEE 841 o equivalente)</t>
-        </is>
-      </c>
-      <c r="C84" s="61" t="n"/>
-      <c r="D84" s="61" t="n"/>
-      <c r="E84" s="61" t="n"/>
-      <c r="F84" s="61" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="60" t="inlineStr">
-        <is>
-          <t>Velocidad</t>
-        </is>
-      </c>
-      <c r="B85" s="60" t="inlineStr">
-        <is>
-          <t>1 800 RPM (4 polos, 60 Hz) — dato típico</t>
-        </is>
-      </c>
-      <c r="C85" s="61" t="n"/>
-      <c r="D85" s="61" t="n"/>
-      <c r="E85" s="61" t="n"/>
-      <c r="F85" s="61" t="n"/>
-    </row>
+      <c r="A82" s="65" t="inlineStr">
+        <is>
+          <t>Referencias de especificación: Leeson/Regal Severe Duty (PDF) (https://www.regalrexnord.com/-/media/documents/brands/literature/industries/leeson_product_catalog_1050.pdf); Baldor-Reliance IEEE 841XL (https://www.baldor.com/mvc/DownloadCenter/Files/9AKK108319) (consulta 2026-07-23).</t>
+        </is>
+      </c>
+    </row>
+    <row r="83"/>
+    <row r="84"/>
     <row r="86">
-      <c r="A86" s="60" t="inlineStr">
-        <is>
-          <t>Aislamiento / protección</t>
-        </is>
-      </c>
-      <c r="B86" s="60" t="inlineStr">
-        <is>
-          <t>Clase F / IP55 mínimo (IP56 preferible)</t>
-        </is>
-      </c>
-      <c r="C86" s="61" t="n"/>
-      <c r="D86" s="61" t="n"/>
-      <c r="E86" s="61" t="n"/>
-      <c r="F86" s="61" t="n"/>
+      <c r="A86" s="62" t="inlineStr">
+        <is>
+          <t>6. Accesorios</t>
+        </is>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" s="60" t="inlineStr">
-        <is>
-          <t>Tensión / fases / frecuencia</t>
-        </is>
-      </c>
-      <c r="B87" s="60" t="inlineStr">
-        <is>
-          <t>440 V, 3φ, 60 Hz (confirmado por el cliente, 2026-07-23)</t>
-        </is>
-      </c>
-      <c r="C87" s="61" t="n"/>
-      <c r="D87" s="61" t="n"/>
-      <c r="E87" s="61" t="n"/>
-      <c r="F87" s="61" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="60" t="inlineStr">
-        <is>
-          <t>Derateo por altitud</t>
-        </is>
-      </c>
-      <c r="B88" s="60" t="inlineStr">
-        <is>
-          <t>≈9 % (NEMA MG-1); absorbido por el margen de selección (§3.2)</t>
-        </is>
-      </c>
-      <c r="C88" s="61" t="n"/>
-      <c r="D88" s="61" t="n"/>
-      <c r="E88" s="61" t="n"/>
-      <c r="F88" s="61" t="n"/>
-    </row>
+      <c r="A87" s="63" t="inlineStr">
+        <is>
+          <t>6.1. Conexión flexible de descarga en hipalón (CSM) con bandas inox 316 (Hardcast Hypalon (PDF) (https://6c2bd45d09da3c66a408-2b16a407535c695c8a76f8b06a56f342.ssl.cf2.rackcdn.com/GWB%20%20eCatalog%2006-25-16.pdf), consulta 2026-07-23).</t>
+        </is>
+      </c>
+    </row>
+    <row r="88"/>
     <row r="89">
-      <c r="A89" s="60" t="inlineStr">
-        <is>
-          <t>Accesorios</t>
-        </is>
-      </c>
-      <c r="B89" s="60" t="inlineStr">
-        <is>
-          <t>Calentador anticondensación si hay paradas largas (dato típico de buena práctica); caja de conexiones sellada, prensaestopas niquelados</t>
-        </is>
-      </c>
-      <c r="C89" s="61" t="n"/>
-      <c r="D89" s="61" t="n"/>
-      <c r="E89" s="61" t="n"/>
-      <c r="F89" s="61" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="63" t="inlineStr">
-        <is>
-          <t>Referencias de especificación: Leeson/Regal Severe Duty (PDF) (https://www.regalrexnord.com/-/media/documents/brands/literature/industries/leeson_product_catalog_1050.pdf); Baldor-Reliance IEEE 841XL (https://www.baldor.com/mvc/DownloadCenter/Files/9AKK108319) (consulta 2026-07-23).</t>
-        </is>
-      </c>
-    </row>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
+      <c r="A89" s="63" t="inlineStr">
+        <is>
+          <t>6.2. Bancada y soportes con ferretería inox 316 (A4) y aislamiento dieléctrico frente a estructura galvanizada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="63" t="inlineStr">
+        <is>
+          <t>6.3. Toma de aire ubicada a sotavento y alejada de las fuentes de cloro de la planta (recomendación de la investigación).</t>
+        </is>
+      </c>
+    </row>
+    <row r="91"/>
+    <row r="92">
+      <c r="A92" s="63" t="inlineStr">
+        <is>
+          <t>6.4. Guardamotor y tablero conforme a RETIE (ver listado_equipos.md, ítems 16-17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="62" t="inlineStr">
+        <is>
+          <t>7. Candidatos comerciales</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="64" t="inlineStr">
+        <is>
+          <t>Tabla 5. Candidatos (consulta 2026-07-23); tamaño/RPM final por confirmar con proveedor.</t>
+        </is>
+      </c>
+    </row>
     <row r="96">
-      <c r="A96" s="62" t="inlineStr">
-        <is>
-          <t>6. Accesorios</t>
-        </is>
-      </c>
+      <c r="A96" s="59" t="inlineStr">
+        <is>
+          <t>Fabricante / línea</t>
+        </is>
+      </c>
+      <c r="B96" s="59" t="n"/>
+      <c r="C96" s="59" t="n"/>
+      <c r="D96" s="59" t="n"/>
+      <c r="E96" s="59" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="F96" s="59" t="n"/>
+      <c r="G96" s="59" t="n"/>
+      <c r="H96" s="59" t="n"/>
+      <c r="I96" s="59" t="inlineStr">
+        <is>
+          <t>Canal en Colombia</t>
+        </is>
+      </c>
+      <c r="J96" s="59" t="n"/>
+      <c r="K96" s="59" t="n"/>
+      <c r="L96" s="59" t="n"/>
+      <c r="M96" s="59" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="N96" s="59" t="n"/>
+      <c r="O96" s="59" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="63" t="inlineStr">
-        <is>
-          <t>6.1. Conexión flexible de descarga en hipalón (CSM) con bandas inox 316 (Hardcast Hypalon (PDF) (https://6c2bd45d09da3c66a408-2b16a407535c695c8a76f8b06a56f342.ssl.cf2.rackcdn.com/GWB%20%20eCatalog%2006-25-16.pdf), consulta 2026-07-23). 6.2. Bancada y soportes con ferretería inox 316 (A4) y aislamiento dieléctrico frente a estructura galvanizada. 6.3. Toma de aire ubicada a sotavento y alejada de las fuentes de cloro de la planta (recomendación de la investigación). 6.4. Guardamotor y tablero conforme a RETIE (ver listado_equipos.md, ítems 16-17).</t>
-        </is>
-      </c>
-    </row>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
+      <c r="A97" s="60" t="inlineStr">
+        <is>
+          <t>Greenheck BCSW-FRP (primera opción)</t>
+        </is>
+      </c>
+      <c r="B97" s="61" t="n"/>
+      <c r="C97" s="61" t="n"/>
+      <c r="D97" s="61" t="n"/>
+      <c r="E97" s="60" t="inlineStr">
+        <is>
+          <t>PRFV poliéster ignífugo, opción velo Nexus</t>
+        </is>
+      </c>
+      <c r="F97" s="61" t="n"/>
+      <c r="G97" s="61" t="n"/>
+      <c r="H97" s="61" t="n"/>
+      <c r="I97" s="60" t="inlineStr">
+        <is>
+          <t>Prime Lines HVAC, Bogotá (representante oficial)</t>
+        </is>
+      </c>
+      <c r="J97" s="61" t="n"/>
+      <c r="K97" s="61" t="n"/>
+      <c r="L97" s="61" t="n"/>
+      <c r="M97" s="60" t="inlineStr">
+        <is>
+          <t>Catálogo (https://content.greenheck.com/public/DAMProd/Original/10002/BCSWFRP_catalog.pdf); rep. (https://www.greenheck.com/find-my-rep/2973_southamerica_colombia)</t>
+        </is>
+      </c>
+      <c r="N97" s="61" t="n"/>
+      <c r="O97" s="61" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="60" t="inlineStr">
+        <is>
+          <t>New York Blower FRP Fume Exhauster</t>
+        </is>
+      </c>
+      <c r="B98" s="61" t="n"/>
+      <c r="C98" s="61" t="n"/>
+      <c r="D98" s="61" t="n"/>
+      <c r="E98" s="60" t="inlineStr">
+        <is>
+          <t>Rueda viniléster PRFV</t>
+        </is>
+      </c>
+      <c r="F98" s="61" t="n"/>
+      <c r="G98" s="61" t="n"/>
+      <c r="H98" s="61" t="n"/>
+      <c r="I98" s="60" t="inlineStr">
+        <is>
+          <t>Importación (plazo máx. ~3 meses, dato cliente 2026-07-23)</t>
+        </is>
+      </c>
+      <c r="J98" s="61" t="n"/>
+      <c r="K98" s="61" t="n"/>
+      <c r="L98" s="61" t="n"/>
+      <c r="M98" s="60" t="inlineStr">
+        <is>
+          <t>NYB (https://www.nyb.com/frp-fume-exhauster/)</t>
+        </is>
+      </c>
+      <c r="N98" s="61" t="n"/>
+      <c r="O98" s="61" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="60" t="inlineStr">
+        <is>
+          <t>Sodeca CPV</t>
+        </is>
+      </c>
+      <c r="B99" s="61" t="n"/>
+      <c r="C99" s="61" t="n"/>
+      <c r="D99" s="61" t="n"/>
+      <c r="E99" s="60" t="inlineStr">
+        <is>
+          <t>Polipropileno</t>
+        </is>
+      </c>
+      <c r="F99" s="61" t="n"/>
+      <c r="G99" s="61" t="n"/>
+      <c r="H99" s="61" t="n"/>
+      <c r="I99" s="60" t="inlineStr">
+        <is>
+          <t>Sodeca Colombia (filial, catálogo 60 Hz)</t>
+        </is>
+      </c>
+      <c r="J99" s="61" t="n"/>
+      <c r="K99" s="61" t="n"/>
+      <c r="L99" s="61" t="n"/>
+      <c r="M99" s="60" t="inlineStr">
+        <is>
+          <t>CPV (https://www.sodeca.com/es/sistemas-de-ventilacion-extraccion/cpv-p1000000071)</t>
+        </is>
+      </c>
+      <c r="N99" s="61" t="n"/>
+      <c r="O99" s="61" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="60" t="inlineStr">
+        <is>
+          <t>Plastec 25/30</t>
+        </is>
+      </c>
+      <c r="B100" s="61" t="n"/>
+      <c r="C100" s="61" t="n"/>
+      <c r="D100" s="61" t="n"/>
+      <c r="E100" s="60" t="inlineStr">
+        <is>
+          <t>Polipropileno, sin metal en corriente</t>
+        </is>
+      </c>
+      <c r="F100" s="61" t="n"/>
+      <c r="G100" s="61" t="n"/>
+      <c r="H100" s="61" t="n"/>
+      <c r="I100" s="60" t="inlineStr">
+        <is>
+          <t>Importación directa (despacho 48 h declarado)</t>
+        </is>
+      </c>
+      <c r="J100" s="61" t="n"/>
+      <c r="K100" s="61" t="n"/>
+      <c r="L100" s="61" t="n"/>
+      <c r="M100" s="60" t="inlineStr">
+        <is>
+          <t>Plastec (https://www.plastecventilation.com/collections/plastec-series)</t>
+        </is>
+      </c>
+      <c r="N100" s="61" t="n"/>
+      <c r="O100" s="61" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="60" t="inlineStr">
+        <is>
+          <t>Soler &amp; Palau línea PP</t>
+        </is>
+      </c>
+      <c r="B101" s="61" t="n"/>
+      <c r="C101" s="61" t="n"/>
+      <c r="D101" s="61" t="n"/>
+      <c r="E101" s="60" t="inlineStr">
+        <is>
+          <t>Polipropileno</t>
+        </is>
+      </c>
+      <c r="F101" s="61" t="n"/>
+      <c r="G101" s="61" t="n"/>
+      <c r="H101" s="61" t="n"/>
+      <c r="I101" s="60" t="inlineStr">
+        <is>
+          <t>S&amp;P Colombia (filial); modelo por confirmar</t>
+        </is>
+      </c>
+      <c r="J101" s="61" t="n"/>
+      <c r="K101" s="61" t="n"/>
+      <c r="L101" s="61" t="n"/>
+      <c r="M101" s="60" t="inlineStr">
+        <is>
+          <t>Catálogo Industrial (PDF) (https://www.solerpalau.mx/ASW/recursos/cata/Industrial.pdf)</t>
+        </is>
+      </c>
+      <c r="N101" s="61" t="n"/>
+      <c r="O101" s="61" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="62" t="inlineStr">
+        <is>
+          <t>8. Normas aplicables</t>
+        </is>
+      </c>
+    </row>
     <row r="105">
-      <c r="A105" s="62" t="inlineStr">
-        <is>
-          <t>7. Candidatos comerciales</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="64" t="inlineStr">
-        <is>
-          <t>Tabla 5. Candidatos (consulta 2026-07-23); tamaño/RPM final por confirmar con proveedor.</t>
-        </is>
-      </c>
-    </row>
+      <c r="A105" s="63" t="inlineStr">
+        <is>
+          <t>8.1. AMCA 210/211 (desempeño y certificación), AMCA 99 (Spark A), ASTM C582 y ASTM D4167 (laminados PRFV), NEMA MG-1 / IEC 60034-1 (motores y derateo por altitud), IEEE 841 (ejecución severe duty de referencia), RETIE y NTC 2050 (instalación eléctrica), ISO 12944 / prácticas NACE-AMPP (protección anticorrosiva del entorno de instalación).</t>
+        </is>
+      </c>
+    </row>
+    <row r="106"/>
     <row r="107"/>
     <row r="108">
-      <c r="A108" s="59" t="inlineStr">
-        <is>
-          <t>Fabricante / línea</t>
-        </is>
-      </c>
-      <c r="B108" s="59" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="C108" s="59" t="inlineStr">
-        <is>
-          <t>Canal en Colombia</t>
-        </is>
-      </c>
-      <c r="D108" s="59" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="E108" s="59" t="n"/>
-      <c r="F108" s="59" t="n"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="60" t="inlineStr">
-        <is>
-          <t>Greenheck BCSW-FRP (primera opción)</t>
-        </is>
-      </c>
-      <c r="B109" s="60" t="inlineStr">
-        <is>
-          <t>PRFV poliéster ignífugo, opción velo Nexus</t>
-        </is>
-      </c>
-      <c r="C109" s="60" t="inlineStr">
-        <is>
-          <t>Prime Lines HVAC, Bogotá (representante oficial)</t>
-        </is>
-      </c>
-      <c r="D109" s="60" t="inlineStr">
-        <is>
-          <t>Catálogo (https://content.greenheck.com/public/DAMProd/Original/10002/BCSWFRP_catalog.pdf); rep. (https://www.greenheck.com/find-my-rep/2973_southamerica_colombia)</t>
-        </is>
-      </c>
-      <c r="E109" s="61" t="n"/>
-      <c r="F109" s="61" t="n"/>
-    </row>
-    <row r="110">
-      <c r="A110" s="60" t="inlineStr">
-        <is>
-          <t>New York Blower FRP Fume Exhauster</t>
-        </is>
-      </c>
-      <c r="B110" s="60" t="inlineStr">
-        <is>
-          <t>Rueda viniléster PRFV</t>
-        </is>
-      </c>
-      <c r="C110" s="60" t="inlineStr">
-        <is>
-          <t>Importación (plazo máx. ~3 meses, dato cliente 2026-07-23)</t>
-        </is>
-      </c>
-      <c r="D110" s="60" t="inlineStr">
-        <is>
-          <t>NYB (https://www.nyb.com/frp-fume-exhauster/)</t>
-        </is>
-      </c>
-      <c r="E110" s="61" t="n"/>
-      <c r="F110" s="61" t="n"/>
-    </row>
-    <row r="111">
-      <c r="A111" s="60" t="inlineStr">
-        <is>
-          <t>Sodeca CPV</t>
-        </is>
-      </c>
-      <c r="B111" s="60" t="inlineStr">
-        <is>
-          <t>Polipropileno</t>
-        </is>
-      </c>
-      <c r="C111" s="60" t="inlineStr">
-        <is>
-          <t>Sodeca Colombia (filial, catálogo 60 Hz)</t>
-        </is>
-      </c>
-      <c r="D111" s="60" t="inlineStr">
-        <is>
-          <t>CPV (https://www.sodeca.com/es/sistemas-de-ventilacion-extraccion/cpv-p1000000071)</t>
-        </is>
-      </c>
-      <c r="E111" s="61" t="n"/>
-      <c r="F111" s="61" t="n"/>
-    </row>
-    <row r="112">
-      <c r="A112" s="60" t="inlineStr">
-        <is>
-          <t>Plastec 25/30</t>
-        </is>
-      </c>
-      <c r="B112" s="60" t="inlineStr">
-        <is>
-          <t>Polipropileno, sin metal en corriente</t>
-        </is>
-      </c>
-      <c r="C112" s="60" t="inlineStr">
-        <is>
-          <t>Importación directa (despacho 48 h declarado)</t>
-        </is>
-      </c>
-      <c r="D112" s="60" t="inlineStr">
-        <is>
-          <t>Plastec (https://www.plastecventilation.com/collections/plastec-series)</t>
-        </is>
-      </c>
-      <c r="E112" s="61" t="n"/>
-      <c r="F112" s="61" t="n"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="60" t="inlineStr">
-        <is>
-          <t>Soler &amp; Palau línea PP</t>
-        </is>
-      </c>
-      <c r="B113" s="60" t="inlineStr">
-        <is>
-          <t>Polipropileno</t>
-        </is>
-      </c>
-      <c r="C113" s="60" t="inlineStr">
-        <is>
-          <t>S&amp;P Colombia (filial); modelo por confirmar</t>
-        </is>
-      </c>
-      <c r="D113" s="60" t="inlineStr">
-        <is>
-          <t>Catálogo Industrial (PDF) (https://www.solerpalau.mx/ASW/recursos/cata/Industrial.pdf)</t>
-        </is>
-      </c>
-      <c r="E113" s="61" t="n"/>
-      <c r="F113" s="61" t="n"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="62" t="inlineStr">
-        <is>
-          <t>8. Normas aplicables</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="63" t="inlineStr">
-        <is>
-          <t>8.1. AMCA 210/211 (desempeño y certificación), AMCA 99 (Spark A), ASTM C582 y ASTM D4167 (laminados PRFV), NEMA MG-1 / IEC 60034-1 (motores y derateo por altitud), IEEE 841 (ejecución severe duty de referencia), RETIE y NTC 2050 (instalación eléctrica), ISO 12944 / prácticas NACE-AMPP (protección anticorrosiva del entorno de instalación).</t>
-        </is>
-      </c>
-    </row>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
+      <c r="A108" s="62" t="inlineStr">
+        <is>
+          <t>Referencia gráfica</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="15" customHeight="1"/>
+    <row r="111" ht="15" customHeight="1"/>
+    <row r="112" ht="15" customHeight="1"/>
+    <row r="113" ht="15" customHeight="1"/>
+    <row r="114" ht="15" customHeight="1"/>
+    <row r="115" ht="15" customHeight="1"/>
+    <row r="116" ht="15" customHeight="1"/>
+    <row r="117" ht="15" customHeight="1"/>
+    <row r="118" ht="15" customHeight="1"/>
+    <row r="119" ht="15" customHeight="1"/>
+    <row r="120" ht="15" customHeight="1"/>
+    <row r="121" ht="15" customHeight="1"/>
+    <row r="122" ht="15" customHeight="1"/>
+    <row r="123" ht="15" customHeight="1"/>
+    <row r="124" ht="15" customHeight="1"/>
+    <row r="125" ht="15" customHeight="1"/>
+    <row r="126" ht="15" customHeight="1"/>
+    <row r="127" ht="15" customHeight="1"/>
+    <row r="128" ht="15" customHeight="1"/>
+    <row r="129" ht="15" customHeight="1"/>
+    <row r="130" ht="15" customHeight="1"/>
+    <row r="131" ht="15" customHeight="1"/>
+    <row r="132" ht="15" customHeight="1"/>
+    <row r="133" ht="15" customHeight="1"/>
+    <row r="134" ht="15" customHeight="1"/>
+    <row r="135" ht="15" customHeight="1"/>
+    <row r="136" ht="15" customHeight="1"/>
+    <row r="137" ht="15" customHeight="1"/>
+    <row r="138" ht="15" customHeight="1"/>
+    <row r="139" ht="15" customHeight="1"/>
+    <row r="140" ht="15" customHeight="1"/>
+    <row r="141" ht="15" customHeight="1"/>
+    <row r="142" ht="15" customHeight="1"/>
+    <row r="143" ht="15" customHeight="1"/>
+    <row r="144" ht="15" customHeight="1"/>
+    <row r="145" ht="15" customHeight="1"/>
+    <row r="146" ht="15" customHeight="1"/>
+    <row r="147" ht="15" customHeight="1"/>
+    <row r="148" ht="15" customHeight="1"/>
+    <row r="149" ht="15" customHeight="1"/>
+    <row r="150" ht="15" customHeight="1"/>
+    <row r="151" ht="15" customHeight="1"/>
   </sheetData>
-  <mergeCells count="73">
-    <mergeCell ref="C48:F48"/>
-    <mergeCell ref="A19:F22"/>
-    <mergeCell ref="A106:F107"/>
-    <mergeCell ref="A80:F80"/>
-    <mergeCell ref="A27:F27"/>
-    <mergeCell ref="B66:F66"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="A105:F105"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A28:F29"/>
-    <mergeCell ref="B70:F70"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="D112:F112"/>
+  <mergeCells count="133">
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A25:O25"/>
+    <mergeCell ref="A77:H77"/>
+    <mergeCell ref="A97:D97"/>
+    <mergeCell ref="A50:O52"/>
+    <mergeCell ref="E97:H97"/>
     <mergeCell ref="N3:O3"/>
-    <mergeCell ref="A40:F41"/>
-    <mergeCell ref="B86:F86"/>
-    <mergeCell ref="A116:F116"/>
-    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="A104:O104"/>
+    <mergeCell ref="E96:H96"/>
+    <mergeCell ref="I30:O30"/>
+    <mergeCell ref="K41:O41"/>
+    <mergeCell ref="I77:O77"/>
+    <mergeCell ref="A75:H75"/>
+    <mergeCell ref="N5:O5"/>
+    <mergeCell ref="C2:L3"/>
+    <mergeCell ref="I80:O80"/>
+    <mergeCell ref="E98:H98"/>
+    <mergeCell ref="I61:O61"/>
+    <mergeCell ref="K43:O43"/>
+    <mergeCell ref="A90:O91"/>
+    <mergeCell ref="I57:O57"/>
+    <mergeCell ref="A87:O88"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="I32:O32"/>
+    <mergeCell ref="A99:D99"/>
+    <mergeCell ref="F39:J39"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="I56:O56"/>
+    <mergeCell ref="A101:D101"/>
+    <mergeCell ref="E99:H99"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="B1:B5"/>
+    <mergeCell ref="A58:H58"/>
+    <mergeCell ref="A46:O49"/>
+    <mergeCell ref="I33:O33"/>
+    <mergeCell ref="A82:O84"/>
+    <mergeCell ref="E101:H101"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A73:H73"/>
+    <mergeCell ref="A108:O108"/>
+    <mergeCell ref="A60:H60"/>
+    <mergeCell ref="E100:H100"/>
+    <mergeCell ref="I10:O10"/>
+    <mergeCell ref="A18:O18"/>
+    <mergeCell ref="I59:O59"/>
+    <mergeCell ref="A86:O86"/>
+    <mergeCell ref="I60:O60"/>
+    <mergeCell ref="I74:O74"/>
     <mergeCell ref="N2:O2"/>
-    <mergeCell ref="B67:F67"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="N5:O5"/>
-    <mergeCell ref="C42:F42"/>
-    <mergeCell ref="A96:F96"/>
+    <mergeCell ref="K44:O44"/>
+    <mergeCell ref="F41:J41"/>
+    <mergeCell ref="M97:O97"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A98:D98"/>
+    <mergeCell ref="K40:O40"/>
+    <mergeCell ref="I11:O11"/>
+    <mergeCell ref="I28:O28"/>
+    <mergeCell ref="A62:H62"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="I96:L96"/>
+    <mergeCell ref="N6:O6"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="I62:O62"/>
+    <mergeCell ref="A40:E40"/>
+    <mergeCell ref="I98:L98"/>
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A54:O54"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="M99:O99"/>
+    <mergeCell ref="A100:D100"/>
+    <mergeCell ref="I79:O79"/>
+    <mergeCell ref="I73:O73"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="A61:H61"/>
+    <mergeCell ref="F40:J40"/>
+    <mergeCell ref="I63:O63"/>
+    <mergeCell ref="A65:O69"/>
+    <mergeCell ref="I99:L99"/>
+    <mergeCell ref="A105:O107"/>
+    <mergeCell ref="A74:H74"/>
+    <mergeCell ref="A56:H56"/>
+    <mergeCell ref="I27:O27"/>
+    <mergeCell ref="F38:J38"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A76:H76"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="I76:O76"/>
+    <mergeCell ref="M96:O96"/>
+    <mergeCell ref="A1:A5"/>
+    <mergeCell ref="A9:O9"/>
+    <mergeCell ref="C1:L1"/>
+    <mergeCell ref="K39:O39"/>
+    <mergeCell ref="I97:L97"/>
+    <mergeCell ref="I75:O75"/>
+    <mergeCell ref="A19:O21"/>
+    <mergeCell ref="M98:O98"/>
+    <mergeCell ref="A36:O36"/>
+    <mergeCell ref="K38:O38"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A63:H63"/>
+    <mergeCell ref="A94:O94"/>
+    <mergeCell ref="I12:O12"/>
+    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="F44:J44"/>
+    <mergeCell ref="I14:O14"/>
+    <mergeCell ref="A96:D96"/>
+    <mergeCell ref="I29:O29"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="I78:O78"/>
+    <mergeCell ref="I13:O13"/>
+    <mergeCell ref="A78:H78"/>
+    <mergeCell ref="I31:O31"/>
+    <mergeCell ref="A71:O71"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="M101:O101"/>
+    <mergeCell ref="F42:J42"/>
+    <mergeCell ref="I15:O15"/>
+    <mergeCell ref="A80:H80"/>
     <mergeCell ref="N1:O1"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B88:F88"/>
-    <mergeCell ref="C2:L3"/>
-    <mergeCell ref="B82:F82"/>
-    <mergeCell ref="D113:F113"/>
-    <mergeCell ref="A23:F25"/>
-    <mergeCell ref="C45:F45"/>
-    <mergeCell ref="B69:F69"/>
-    <mergeCell ref="B87:F87"/>
-    <mergeCell ref="B34:F34"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="A72:F78"/>
-    <mergeCell ref="D110:F110"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A56:F59"/>
-    <mergeCell ref="C47:F47"/>
-    <mergeCell ref="B84:F84"/>
-    <mergeCell ref="A39:F39"/>
-    <mergeCell ref="A1:A5"/>
-    <mergeCell ref="C1:L1"/>
-    <mergeCell ref="D109:F109"/>
-    <mergeCell ref="C44:F44"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B65:F65"/>
-    <mergeCell ref="A50:F55"/>
-    <mergeCell ref="B68:F68"/>
-    <mergeCell ref="B83:F83"/>
-    <mergeCell ref="A97:F103"/>
-    <mergeCell ref="A117:F121"/>
-    <mergeCell ref="B64:F64"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="C43:F43"/>
-    <mergeCell ref="B89:F89"/>
+    <mergeCell ref="M100:O100"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="I101:L101"/>
+    <mergeCell ref="A57:H57"/>
+    <mergeCell ref="K42:O42"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="I100:L100"/>
+    <mergeCell ref="F43:J43"/>
     <mergeCell ref="C4:L6"/>
-    <mergeCell ref="N6:O6"/>
-    <mergeCell ref="C46:F46"/>
-    <mergeCell ref="A61:F61"/>
-    <mergeCell ref="D111:F111"/>
-    <mergeCell ref="B63:F63"/>
-    <mergeCell ref="B85:F85"/>
-    <mergeCell ref="B36:F36"/>
-    <mergeCell ref="D108:F108"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="A91:F94"/>
-    <mergeCell ref="B1:B5"/>
-    <mergeCell ref="N4:O4"/>
-    <mergeCell ref="B35:F35"/>
+    <mergeCell ref="I58:O58"/>
+    <mergeCell ref="A22:O23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>